<commit_message>
Add ServiceNow group managers, members, and designations.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/agent_groups/sandbox/empty-cwt-groups-servicenow.xlsx
+++ b/agent_groups/sandbox/empty-cwt-groups-servicenow.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Empty CWT groups" sheetId="1" r:id="rId1"/>
+    <sheet name="Groups" sheetId="1" r:id="rId1"/>
+    <sheet name="Members" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +416,12 @@
       <c r="E1" t="str">
         <v>Active</v>
       </c>
+      <c r="F1" t="str">
+        <v>Group manager</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Member count</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,6 +439,12 @@
       <c r="E2" t="str">
         <v>No</v>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -449,6 +462,12 @@
       <c r="E3" t="str">
         <v>No</v>
       </c>
+      <c r="F3" t="str">
+        <v>Christian Wolff</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -466,6 +485,12 @@
       <c r="E4" t="str">
         <v>No</v>
       </c>
+      <c r="F4" t="str">
+        <v>Ishay Koplovich</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -483,6 +508,12 @@
       <c r="E5" t="str">
         <v>No</v>
       </c>
+      <c r="F5" t="str">
+        <v>Alexander Oelkers</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -500,6 +531,12 @@
       <c r="E6" t="str">
         <v>No</v>
       </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -517,6 +554,12 @@
       <c r="E7" t="str">
         <v>No</v>
       </c>
+      <c r="F7" t="str">
+        <v>Geoffrey Gemoto</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -534,6 +577,12 @@
       <c r="E8" t="str">
         <v>No</v>
       </c>
+      <c r="F8" t="str">
+        <v>Monika Singh</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -551,6 +600,12 @@
       <c r="E9" t="str">
         <v>No</v>
       </c>
+      <c r="F9" t="str">
+        <v>Rajath Kumar</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -568,6 +623,12 @@
       <c r="E10" t="str">
         <v>No</v>
       </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -585,6 +646,12 @@
       <c r="E11" t="str">
         <v>No</v>
       </c>
+      <c r="F11" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="G11">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -602,6 +669,12 @@
       <c r="E12" t="str">
         <v>Yes</v>
       </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -619,10 +692,443 @@
       <c r="E13" t="str">
         <v/>
       </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H16"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Freshservice sandbox</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ServiceNow group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Group manager</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Member name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Designation</v>
+      </c>
+      <c r="G1" t="str">
+        <v>User active</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Note</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>CWT AGM Support</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AGM Support</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CWT DACH Rail</v>
+      </c>
+      <c r="B3" t="str">
+        <v>DACH Rail</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Christian Wolff</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>CWT Digital Security</v>
+      </c>
+      <c r="B4" t="str">
+        <v>CWT Digital Security</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Ishay Koplovich</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CWT EIT DnA Platform Admin L3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CWT EIT DnA Platform Admin L3</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Alexander Oelkers</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Regina Gendler</v>
+      </c>
+      <c r="E5" t="str">
+        <v>regina.gendler@amexgbt.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Application Support Analyst</v>
+      </c>
+      <c r="G5" t="str">
+        <v>true</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CWT EIT DnA Platform Admin L3</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CWT EIT DnA Platform Admin L3</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Alexander Oelkers</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Alexander Oelkers</v>
+      </c>
+      <c r="E6" t="str">
+        <v>alexander.oelkers@amexgbt.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Lead Applications Support</v>
+      </c>
+      <c r="G6" t="str">
+        <v>true</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>CWT FTS ENG NORAM</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FTS ENG NORAM</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CWT GSD Connect Support</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GSD Connect Support</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Geoffrey Gemoto</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>CWT India Products</v>
+      </c>
+      <c r="B9" t="str">
+        <v>CWT India Products</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Monika Singh</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Monika Singh</v>
+      </c>
+      <c r="E9" t="str">
+        <v>monika.singh1@amexgbt.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Manager II, Global Product Optimisation</v>
+      </c>
+      <c r="G9" t="str">
+        <v>true</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>CWT INTERACTION PLATFORMS ASIA PAC</v>
+      </c>
+      <c r="B10" t="str">
+        <v>INTERACTION PLATFORMS ASIA PAC</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Rajath Kumar</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>CWT Security Operations</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Security Operations</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>CWT TXC L2 CWT Resolve</v>
+      </c>
+      <c r="B12" t="str">
+        <v>TXC L2 CWT Resolve</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Esmeralda Perez</v>
+      </c>
+      <c r="E12" t="str">
+        <v>esmeralda.perez@amexgbt.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Desktop Configuration Specialist II</v>
+      </c>
+      <c r="G12" t="str">
+        <v>true</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>CWT TXC L2 CWT Resolve</v>
+      </c>
+      <c r="B13" t="str">
+        <v>TXC L2 CWT Resolve</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Aislinn Millan</v>
+      </c>
+      <c r="E13" t="str">
+        <v>aislinn.millan@amexgbt.com</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Desktop Configuration Specialist II</v>
+      </c>
+      <c r="G13" t="str">
+        <v>true</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>CWT TXC L2 CWT Resolve</v>
+      </c>
+      <c r="B14" t="str">
+        <v>TXC L2 CWT Resolve</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Ana Maria Perez Ayuso</v>
+      </c>
+      <c r="E14" t="str">
+        <v>anamaria.perezayuso@amexgbt.com</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Desktop Configuration Specialist II</v>
+      </c>
+      <c r="G14" t="str">
+        <v>true</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>CWT TXC L2 CWT Resolve</v>
+      </c>
+      <c r="B15" t="str">
+        <v>TXC L2 CWT Resolve</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Katarina Exerman</v>
+      </c>
+      <c r="E15" t="str">
+        <v>katarina.exerman@amexgbt.com</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Senior Manager, Desktop Configuration</v>
+      </c>
+      <c r="G15" t="str">
+        <v>true</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CWT Work Force Management (WFM)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Work Force Management  (WFM)</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>No members</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>